<commit_message>
Adding UI Changes for APP
</commit_message>
<xml_diff>
--- a/test-data/Templates/DEV/ATBP.xlsx
+++ b/test-data/Templates/DEV/ATBP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tejavathidoddapaneni/MaextroAutomationTests/test-data/BP Templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tejavathidoddapaneni/Maextro_AutomationApp/test-data/Templates/DEV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4D4099-55C6-8941-ACF6-683CACD55772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D1DA99-0416-564F-8CC7-2E7F4B1A9E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15100" yWindow="660" windowWidth="15140" windowHeight="17180" xr2:uid="{9B722DE1-D4F2-8E4B-A1FC-B7FBF3A04462}"/>
+    <workbookView xWindow="260" yWindow="660" windowWidth="15140" windowHeight="17180" xr2:uid="{9B722DE1-D4F2-8E4B-A1FC-B7FBF3A04462}"/>
   </bookViews>
   <sheets>
     <sheet name="MXT_HDR" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="141">
   <si>
     <t>Object</t>
   </si>
@@ -114,9 +114,6 @@
   </si>
   <si>
     <t>BP08</t>
-  </si>
-  <si>
-    <t>Skip</t>
   </si>
   <si>
     <t>BP No</t>
@@ -912,7 +909,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -963,10 +960,10 @@
         <v>13</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -980,7 +977,7 @@
         <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -991,10 +988,10 @@
         <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -1008,7 +1005,7 @@
         <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -1022,7 +1019,7 @@
         <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>140</v>
       </c>
       <c r="E10" s="3"/>
     </row>
@@ -1037,7 +1034,7 @@
         <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>140</v>
       </c>
       <c r="E11" s="3"/>
     </row>
@@ -1057,6 +1054,20 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D6:D11" xr:uid="{AAFA66C4-3E29-3E44-95AF-5AF2523CFC23}">
+      <formula1>"Save,Skip,Approve,Reject -&gt; Approve"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{F81BD13B-E4A5-A14D-B072-592B59BC0410}">
+      <formula1>"New customer"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{C3A927F9-677E-6C47-AB59-F81F6F5CFE6B}">
+      <formula1>"BSX RDS DIVISION,DEMO DIVISION CODE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{7A3F8F73-F4FE-384D-B132-60A711F27BD8}">
+      <formula1>"Low,Medium,High"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1074,21 +1085,21 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1096,7 +1107,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1104,26 +1115,26 @@
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -1138,24 +1149,24 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -1176,30 +1187,30 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1210,10 +1221,10 @@
         <v>1000</v>
       </c>
       <c r="F18" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G18" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1224,10 +1235,10 @@
         <v>2000</v>
       </c>
       <c r="F19" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1245,21 +1256,21 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
@@ -1274,63 +1285,63 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="L7" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="M7" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="N7" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N7" s="1" t="s">
+      <c r="O7" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O7" s="1" t="s">
+      <c r="P7" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="P7" s="1" t="s">
+      <c r="Q7" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="Q7" s="1" t="s">
+      <c r="R7" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
@@ -1338,49 +1349,49 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" t="s">
         <v>65</v>
       </c>
-      <c r="D8" t="s">
+      <c r="F8" t="s">
         <v>66</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>67</v>
       </c>
-      <c r="G8" t="s">
-        <v>68</v>
-      </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I8">
         <v>15</v>
       </c>
       <c r="J8" t="s">
+        <v>68</v>
+      </c>
+      <c r="K8" t="s">
         <v>69</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>70</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>71</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>72</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>73</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>74</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
         <v>75</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="R8" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="R8" s="5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
@@ -1388,49 +1399,49 @@
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D9" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" t="s">
         <v>78</v>
       </c>
-      <c r="F9" t="s">
-        <v>79</v>
-      </c>
       <c r="G9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I9">
         <v>28</v>
       </c>
       <c r="J9" t="s">
+        <v>79</v>
+      </c>
+      <c r="K9" t="s">
         <v>80</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>81</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
+        <v>71</v>
+      </c>
+      <c r="N9" t="s">
+        <v>72</v>
+      </c>
+      <c r="O9" t="s">
         <v>82</v>
       </c>
-      <c r="M9" t="s">
-        <v>72</v>
-      </c>
-      <c r="N9" t="s">
-        <v>73</v>
-      </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>83</v>
       </c>
-      <c r="P9" t="s">
+      <c r="Q9" t="s">
         <v>84</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" s="5" t="s">
         <v>85</v>
-      </c>
-      <c r="R9" s="5" t="s">
-        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1452,21 +1463,21 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -1481,42 +1492,42 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="K7" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -1524,22 +1535,22 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
+        <v>93</v>
+      </c>
+      <c r="E8" t="s">
         <v>94</v>
-      </c>
-      <c r="E8" t="s">
-        <v>95</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
       <c r="J8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
@@ -1547,50 +1558,50 @@
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
       <c r="J9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="G12" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -1602,16 +1613,16 @@
         <v>1</v>
       </c>
       <c r="D13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E13" t="s">
         <v>103</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>104</v>
       </c>
-      <c r="F13" t="s">
-        <v>105</v>
-      </c>
       <c r="G13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
@@ -1621,16 +1632,16 @@
         <v>2</v>
       </c>
       <c r="D14" t="s">
+        <v>105</v>
+      </c>
+      <c r="E14" t="s">
         <v>106</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>107</v>
       </c>
-      <c r="F14" t="s">
-        <v>108</v>
-      </c>
       <c r="G14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
@@ -1660,57 +1671,57 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -1721,7 +1732,7 @@
         <v>1234567890</v>
       </c>
       <c r="G3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -1732,7 +1743,7 @@
         <v>9876543210</v>
       </c>
       <c r="G4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1750,25 +1761,25 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -1776,16 +1787,16 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E2" t="s">
         <v>103</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>104</v>
       </c>
-      <c r="F2" t="s">
-        <v>105</v>
-      </c>
       <c r="G2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -1793,42 +1804,42 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E3" t="s">
         <v>106</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>107</v>
       </c>
-      <c r="F3" t="s">
-        <v>108</v>
-      </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -1836,13 +1847,13 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
+        <v>129</v>
+      </c>
+      <c r="G6" t="s">
         <v>130</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>131</v>
-      </c>
-      <c r="H6" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -1850,13 +1861,13 @@
         <v>2</v>
       </c>
       <c r="F7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H7" t="s">
         <v>133</v>
-      </c>
-      <c r="H7" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1874,16 +1885,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated UI and functionalities
</commit_message>
<xml_diff>
--- a/test-data/Templates/DEV/ATBP.xlsx
+++ b/test-data/Templates/DEV/ATBP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tejavathidoddapaneni/Maextro_AutomationApp/test-data/Templates/DEV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D1DA99-0416-564F-8CC7-2E7F4B1A9E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FBC6017-79CB-3B49-83AD-334967E7FA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="260" yWindow="660" windowWidth="15140" windowHeight="17180" xr2:uid="{9B722DE1-D4F2-8E4B-A1FC-B7FBF3A04462}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{9B722DE1-D4F2-8E4B-A1FC-B7FBF3A04462}"/>
   </bookViews>
   <sheets>
     <sheet name="MXT_HDR" sheetId="1" r:id="rId1"/>
@@ -874,7 +874,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04F06E39-692B-1A44-8C52-E130C06F25B7}">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.1640625" bestFit="1" customWidth="1"/>
@@ -1038,26 +1038,8 @@
       </c>
       <c r="E11" s="3"/>
     </row>
-    <row r="27" spans="12:12" x14ac:dyDescent="0.2">
-      <c r="L27">
-        <v>39182</v>
-      </c>
-    </row>
-    <row r="29" spans="12:12" x14ac:dyDescent="0.2">
-      <c r="L29">
-        <v>39185</v>
-      </c>
-    </row>
-    <row r="30" spans="12:12" x14ac:dyDescent="0.2">
-      <c r="L30">
-        <v>39186</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D6:D11" xr:uid="{AAFA66C4-3E29-3E44-95AF-5AF2523CFC23}">
-      <formula1>"Save,Skip,Approve,Reject -&gt; Approve"</formula1>
-    </dataValidation>
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{F81BD13B-E4A5-A14D-B072-592B59BC0410}">
       <formula1>"New customer"</formula1>
     </dataValidation>
@@ -1066,6 +1048,9 @@
     </dataValidation>
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{7A3F8F73-F4FE-384D-B132-60A711F27BD8}">
       <formula1>"Low,Medium,High"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D6:D11" xr:uid="{40DEADEC-5B07-D343-8084-14759BD0A5AC}">
+      <formula1>"Save,Skip,Approve,Skip -&gt; Save,Skip -&gt; Approve,Reject -&gt; Approve"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>